<commit_message>
Regenerate Shemot-Devarim 5787 sheets with scrolls and join code
Rebuild the four unposted 5787 workbooks with each book's scroll
(Shemot: Kaufman, Vayikra: Red, Bamidbar: Gunther, Devarim: Gunther)
and Beth Sholom's Virtual Tikkun join code, so every link ends in
&join=24A677PXECFW. Bereshit 5787 is left as is: it is already live
on Google Sheets.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bamidbar 5787.xlsx
+++ b/Bamidbar 5787.xlsx
@@ -2082,11 +2082,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -2123,7 +2123,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -2138,7 +2138,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -2153,7 +2153,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz&amp;aliyah=A3", "III")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz&amp;aliyah=A3&amp;join=24A677PXECFW", "III")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2515,11 +2515,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz (Mincha)", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz (Mincha)&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -2556,7 +2556,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz (Mincha)&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz (Mincha)&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -2571,7 +2571,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz (Mincha)&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz (Mincha)&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -2586,7 +2586,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz (Mincha)&amp;aliyah=M", "Maf")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Tzom Tammuz (Mincha)&amp;aliyah=M&amp;join=24A677PXECFW", "Maf")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2956,11 +2956,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -2997,7 +2997,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -3012,7 +3012,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -3027,7 +3027,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A3", "III")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A3&amp;join=24A677PXECFW", "III")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -3042,7 +3042,7 @@
     </row>
     <row r="18">
       <c r="A18" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A4", "IV")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A4&amp;join=24A677PXECFW", "IV")</f>
         <v/>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -3057,7 +3057,7 @@
     </row>
     <row r="19">
       <c r="A19" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A5", "V")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A5&amp;join=24A677PXECFW", "V")</f>
         <v/>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -3072,7 +3072,7 @@
     </row>
     <row r="20">
       <c r="A20" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A6", "VI")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A6&amp;join=24A677PXECFW", "VI")</f>
         <v/>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -3087,7 +3087,7 @@
     </row>
     <row r="21">
       <c r="A21" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A7", "VII")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=A7&amp;join=24A677PXECFW", "VII")</f>
         <v/>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -3102,7 +3102,7 @@
     </row>
     <row r="22">
       <c r="A22" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=M", "Maf")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Pinchas&amp;aliyah=M&amp;join=24A677PXECFW", "Maf")</f>
         <v/>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -3468,11 +3468,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -3509,7 +3509,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -3524,7 +3524,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -3539,7 +3539,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A3", "III")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A3&amp;join=24A677PXECFW", "III")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -3554,7 +3554,7 @@
     </row>
     <row r="18">
       <c r="A18" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A4", "IV")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A4&amp;join=24A677PXECFW", "IV")</f>
         <v/>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -3569,7 +3569,7 @@
     </row>
     <row r="19">
       <c r="A19" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A5", "V")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A5&amp;join=24A677PXECFW", "V")</f>
         <v/>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -3584,7 +3584,7 @@
     </row>
     <row r="20">
       <c r="A20" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A6", "VI")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A6&amp;join=24A677PXECFW", "VI")</f>
         <v/>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -3599,7 +3599,7 @@
     </row>
     <row r="21">
       <c r="A21" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A7", "VII")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=A7&amp;join=24A677PXECFW", "VII")</f>
         <v/>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -3614,7 +3614,7 @@
     </row>
     <row r="22">
       <c r="A22" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=M", "Maf")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Matot-Masei&amp;aliyah=M&amp;join=24A677PXECFW", "Maf")</f>
         <v/>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -3984,11 +3984,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -4025,7 +4025,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -4040,7 +4040,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -4055,7 +4055,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A3", "III")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A3&amp;join=24A677PXECFW", "III")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -4070,7 +4070,7 @@
     </row>
     <row r="18">
       <c r="A18" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A4", "IV")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A4&amp;join=24A677PXECFW", "IV")</f>
         <v/>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -4085,7 +4085,7 @@
     </row>
     <row r="19">
       <c r="A19" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A5", "V")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A5&amp;join=24A677PXECFW", "V")</f>
         <v/>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -4100,7 +4100,7 @@
     </row>
     <row r="20">
       <c r="A20" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A6", "VI")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A6&amp;join=24A677PXECFW", "VI")</f>
         <v/>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -4115,7 +4115,7 @@
     </row>
     <row r="21">
       <c r="A21" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A7", "VII")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=A7&amp;join=24A677PXECFW", "VII")</f>
         <v/>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -4130,7 +4130,7 @@
     </row>
     <row r="22">
       <c r="A22" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=M", "Maf")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Bamidbar&amp;aliyah=M&amp;join=24A677PXECFW", "Maf")</f>
         <v/>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -4496,11 +4496,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -4537,7 +4537,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -4552,7 +4552,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -4567,7 +4567,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=A3", "III")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=A3&amp;join=24A677PXECFW", "III")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -4582,7 +4582,7 @@
     </row>
     <row r="18">
       <c r="A18" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=A4", "IV")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=A4&amp;join=24A677PXECFW", "IV")</f>
         <v/>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -4597,7 +4597,7 @@
     </row>
     <row r="19">
       <c r="A19" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=A5", "V")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=A5&amp;join=24A677PXECFW", "V")</f>
         <v/>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -4612,7 +4612,7 @@
     </row>
     <row r="20">
       <c r="A20" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=M", "Maf")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot I&amp;aliyah=M&amp;join=24A677PXECFW", "Maf")</f>
         <v/>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -4978,11 +4978,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -5019,7 +5019,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -5034,7 +5034,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -5049,7 +5049,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A3", "III")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A3&amp;join=24A677PXECFW", "III")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -5064,7 +5064,7 @@
     </row>
     <row r="18">
       <c r="A18" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A4", "IV")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A4&amp;join=24A677PXECFW", "IV")</f>
         <v/>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -5079,7 +5079,7 @@
     </row>
     <row r="19">
       <c r="A19" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A5", "V")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A5&amp;join=24A677PXECFW", "V")</f>
         <v/>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -5094,7 +5094,7 @@
     </row>
     <row r="20">
       <c r="A20" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A6", "VI")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A6&amp;join=24A677PXECFW", "VI")</f>
         <v/>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -5109,7 +5109,7 @@
     </row>
     <row r="21">
       <c r="A21" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A7", "VII")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=A7&amp;join=24A677PXECFW", "VII")</f>
         <v/>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -5124,7 +5124,7 @@
     </row>
     <row r="22">
       <c r="A22" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=M", "Maf")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shavuot II (on Shabbat)&amp;aliyah=M&amp;join=24A677PXECFW", "Maf")</f>
         <v/>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -5490,11 +5490,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -5531,7 +5531,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -5546,7 +5546,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -5561,7 +5561,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A3", "III")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A3&amp;join=24A677PXECFW", "III")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -5576,7 +5576,7 @@
     </row>
     <row r="18">
       <c r="A18" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A4", "IV")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A4&amp;join=24A677PXECFW", "IV")</f>
         <v/>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -5591,7 +5591,7 @@
     </row>
     <row r="19">
       <c r="A19" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A5", "V")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A5&amp;join=24A677PXECFW", "V")</f>
         <v/>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -5606,7 +5606,7 @@
     </row>
     <row r="20">
       <c r="A20" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A6", "VI")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A6&amp;join=24A677PXECFW", "VI")</f>
         <v/>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -5621,7 +5621,7 @@
     </row>
     <row r="21">
       <c r="A21" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A7", "VII")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=A7&amp;join=24A677PXECFW", "VII")</f>
         <v/>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -5636,7 +5636,7 @@
     </row>
     <row r="22">
       <c r="A22" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=M", "Maf")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Nasso&amp;aliyah=M&amp;join=24A677PXECFW", "Maf")</f>
         <v/>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -6002,11 +6002,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -6043,7 +6043,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -6058,7 +6058,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -6073,7 +6073,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A3", "III")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A3&amp;join=24A677PXECFW", "III")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -6088,7 +6088,7 @@
     </row>
     <row r="18">
       <c r="A18" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A4", "IV")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A4&amp;join=24A677PXECFW", "IV")</f>
         <v/>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -6103,7 +6103,7 @@
     </row>
     <row r="19">
       <c r="A19" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A5", "V")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A5&amp;join=24A677PXECFW", "V")</f>
         <v/>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -6118,7 +6118,7 @@
     </row>
     <row r="20">
       <c r="A20" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A6", "VI")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A6&amp;join=24A677PXECFW", "VI")</f>
         <v/>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -6133,7 +6133,7 @@
     </row>
     <row r="21">
       <c r="A21" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A7", "VII")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=A7&amp;join=24A677PXECFW", "VII")</f>
         <v/>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -6148,7 +6148,7 @@
     </row>
     <row r="22">
       <c r="A22" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=M", "Maf")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Beha'alotcha&amp;aliyah=M&amp;join=24A677PXECFW", "Maf")</f>
         <v/>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -6514,11 +6514,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -6555,7 +6555,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -6570,7 +6570,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -6585,7 +6585,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A3", "III")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A3&amp;join=24A677PXECFW", "III")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -6600,7 +6600,7 @@
     </row>
     <row r="18">
       <c r="A18" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A4", "IV")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A4&amp;join=24A677PXECFW", "IV")</f>
         <v/>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -6615,7 +6615,7 @@
     </row>
     <row r="19">
       <c r="A19" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A5", "V")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A5&amp;join=24A677PXECFW", "V")</f>
         <v/>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -6630,7 +6630,7 @@
     </row>
     <row r="20">
       <c r="A20" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A6", "VI")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A6&amp;join=24A677PXECFW", "VI")</f>
         <v/>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -6645,7 +6645,7 @@
     </row>
     <row r="21">
       <c r="A21" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A7", "VII")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=A7&amp;join=24A677PXECFW", "VII")</f>
         <v/>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -6660,7 +6660,7 @@
     </row>
     <row r="22">
       <c r="A22" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=M", "Maf")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sh'lach&amp;aliyah=M&amp;join=24A677PXECFW", "Maf")</f>
         <v/>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -7026,11 +7026,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -7067,7 +7067,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -7082,7 +7082,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -7097,7 +7097,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A3", "III")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A3&amp;join=24A677PXECFW", "III")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -7112,7 +7112,7 @@
     </row>
     <row r="18">
       <c r="A18" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A4", "IV")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A4&amp;join=24A677PXECFW", "IV")</f>
         <v/>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -7127,7 +7127,7 @@
     </row>
     <row r="19">
       <c r="A19" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A5", "V")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A5&amp;join=24A677PXECFW", "V")</f>
         <v/>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -7142,7 +7142,7 @@
     </row>
     <row r="20">
       <c r="A20" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A6", "VI")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A6&amp;join=24A677PXECFW", "VI")</f>
         <v/>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -7157,7 +7157,7 @@
     </row>
     <row r="21">
       <c r="A21" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A7", "VII")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=A7&amp;join=24A677PXECFW", "VII")</f>
         <v/>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -7172,7 +7172,7 @@
     </row>
     <row r="22">
       <c r="A22" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=M", "Maf")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Korach&amp;aliyah=M&amp;join=24A677PXECFW", "Maf")</f>
         <v/>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -7538,11 +7538,11 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Gunther</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak", "Virtual Tikkun")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;join=24A677PXECFW", "Virtual Tikkun")</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -7579,7 +7579,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A1", "I")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A1&amp;join=24A677PXECFW", "I")</f>
         <v/>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -7594,7 +7594,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A2", "II")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A2&amp;join=24A677PXECFW", "II")</f>
         <v/>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -7609,7 +7609,7 @@
     </row>
     <row r="17">
       <c r="A17" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A3", "III")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A3&amp;join=24A677PXECFW", "III")</f>
         <v/>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -7624,7 +7624,7 @@
     </row>
     <row r="18">
       <c r="A18" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A4", "IV")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A4&amp;join=24A677PXECFW", "IV")</f>
         <v/>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -7639,7 +7639,7 @@
     </row>
     <row r="19">
       <c r="A19" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A5", "V")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A5&amp;join=24A677PXECFW", "V")</f>
         <v/>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -7654,7 +7654,7 @@
     </row>
     <row r="20">
       <c r="A20" s="13">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A6", "VI")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A6&amp;join=24A677PXECFW", "VI")</f>
         <v/>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -7669,7 +7669,7 @@
     </row>
     <row r="21">
       <c r="A21" s="9">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A7", "VII")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=A7&amp;join=24A677PXECFW", "VII")</f>
         <v/>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -7684,7 +7684,7 @@
     </row>
     <row r="22">
       <c r="A22" s="11">
-        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=M", "Maf")</f>
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Chukat-Balak&amp;aliyah=M&amp;join=24A677PXECFW", "Maf")</f>
         <v/>
       </c>
       <c r="B22" s="12" t="inlineStr">

</xml_diff>